<commit_message>
Created and initialised arrays with artists and songs, data is derived from associated text files
</commit_message>
<xml_diff>
--- a/100 Data assignment/Artist data collection.xlsx
+++ b/100 Data assignment/Artist data collection.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/92370d87bc01a04c/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/92370d87bc01a04c/Documents/Portfolio/100 Data assignment/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="38" documentId="8_{1812C6AA-B58E-4CF3-B398-9FA38DB1BDD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B0C18476-C866-4ADE-AFAD-E3E80A08D4D6}"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -507,28 +507,6 @@
   </cellStyles>
   <dxfs count="6">
     <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
       <border>
         <left style="thin">
           <color auto="1"/>
@@ -578,6 +556,28 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -599,7 +599,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9E23E9EF-C872-DE44-8DAD-6FE065537A9D}" name="Artists" displayName="Artists" ref="A1:F32" totalsRowShown="0">
   <autoFilter ref="A1:F32" xr:uid="{9E23E9EF-C872-DE44-8DAD-6FE065537A9D}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{422E9A63-580E-B74A-A55F-1FF67CDB3711}" name="Day" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{422E9A63-580E-B74A-A55F-1FF67CDB3711}" name="Day" dataDxfId="5"/>
     <tableColumn id="2" xr3:uid="{E33050B7-B8F1-8A49-912E-E11B98FB6652}" name="Artist1"/>
     <tableColumn id="3" xr3:uid="{8FAEF343-35F4-4643-A2A2-1C4EA8808C0F}" name="Artist2"/>
     <tableColumn id="4" xr3:uid="{4448714E-4507-A14E-895D-5B5AB1719F6E}" name="Artist3"/>
@@ -614,7 +614,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{14CA18EF-08D5-B44F-B21F-B8B8339F131E}" name="Songs" displayName="Songs" ref="H1:M32" totalsRowShown="0">
   <autoFilter ref="H1:M32" xr:uid="{14CA18EF-08D5-B44F-B21F-B8B8339F131E}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{CE0F3196-2E60-C342-8722-A66E0B9AB7F4}" name="Day" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{CE0F3196-2E60-C342-8722-A66E0B9AB7F4}" name="Day" dataDxfId="4"/>
     <tableColumn id="2" xr3:uid="{BB445233-ED05-DB43-8DDA-39006BED02CF}" name="Song1"/>
     <tableColumn id="3" xr3:uid="{E0C63A0E-1498-6049-BD4A-E6AE28CE0893}" name="Song2"/>
     <tableColumn id="4" xr3:uid="{CD7582B9-E6C6-F74C-89DC-A20F0AFCD016}" name="Song3"/>
@@ -2305,18 +2305,18 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="O3:P200">
-    <cfRule type="expression" dxfId="5" priority="2">
+    <cfRule type="expression" dxfId="3" priority="2">
       <formula>AND($O3&lt;&gt;"", ISEVEN(ROW()-ROW($O$3)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="3">
+    <cfRule type="expression" dxfId="2" priority="3">
       <formula>$O3&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R3:S200">
-    <cfRule type="expression" dxfId="3" priority="1">
+    <cfRule type="expression" dxfId="1" priority="1">
       <formula>AND($R3&lt;&gt;"", ISEVEN(ROW()-ROW($R$3)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="4" stopIfTrue="1">
+    <cfRule type="expression" dxfId="0" priority="4" stopIfTrue="1">
       <formula>$R3&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>